<commit_message>
feat(F-NAR-019): polish TREE-AUT-015 xlsx
Alignement xlsx sur merged vocal après re-apply.
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-015.xlsx
+++ b/stories/arbres/TREE-AUT-015.xlsx
@@ -3112,17 +3112,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Le ballon dans le sac, et la pomme dans le creux ! Nina souffle, puis avance une main. Elle suit le grain de sel, jusqu'au bouton de bois. Le ballon rentre, la pomme se cale, ronde. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. La pomme a un nid, maintenant ! Le trou a failli tout garder. Une miette de pomme dort dans le sable. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>Le ballon dans le sac, et la pomme dans le creux ! Nina souffle, puis avance une main. Le grain de sel guide sa main, vers le bouton. Le ballon rentre, la pomme se cale, ronde. Le sac se ferme, grain au milieu. Le grain a parlé, très bas. La pomme a un nid, maintenant ! Le trou a failli tout garder. Une miette de pomme dort dans le sable. Le grain est là, tu le sens ? Oui, c'est celui de la buée.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le ballon dans le sac, et la pomme dans le creux ! Nina souffle, puis avance une main. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le ballon rentre, la pomme se cale, ronde. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. La pomme a un nid, maintenant ! Le trou a failli tout garder. Une miette de pomme dort dans le sable. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le ballon dans le sac, et la pomme dans le creux ! Nina souffle, puis avance une main. Le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt; guide sa main, vers le bouton. Le ballon rentre, la pomme se cale, ronde. Le sac se ferme, grain au milieu. Le grain a parlé, très bas. La pomme a un nid, maintenant ! Le trou a failli tout garder. Une miette de pomme dort dans le sable. Le grain est là, tu le sens ? Oui, c'est celui de la buée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Le ballon dans le sac, et la pomme dans le creux ! Nina souffle, puis avance une main. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le ballon rentre, la pomme se cale, ronde. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. La pomme a un nid, maintenant ! Le trou a failli tout garder. Une miette de pomme dort dans le sable. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>Le ballon dans le sac, et la pomme dans le creux ! Nina souffle, puis avance une main. Le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt; guide sa main, vers le bouton. Le ballon rentre, la pomme se cale, ronde. Le sac se ferme, grain au milieu. Le grain a parlé, très bas. La pomme a un nid, maintenant ! Le trou a failli tout garder. Une miette de pomme dort dans le sable. Le grain est là, tu le sens ? Oui, c'est celui de la buée. [pause]</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -3258,15 +3258,15 @@
         <is>
           <t>enfant-f|Le ballon dans le sac, et la pomme dans le creux !
 narrateur|Nina souffle, puis avance une main.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Le grain de sel guide sa main, vers le bouton.
 narrateur|Le ballon rentre, la pomme se cale, ronde.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le sac se ferme, grain au milieu.
 papa|Le grain a parlé, très bas.
 enfant-f|La pomme a un nid, maintenant !
 maman|Le trou a failli tout garder.
 narrateur|Une miette de pomme dort dans le sable.
-papa|Tu as vu le grain, sur le bouton ?
-enfant-f|Il était sur la vitre, à la cuisine.</t>
+papa|Le grain est là, tu le sens ?
+enfant-f|Oui, c'est celui de la buée.</t>
         </is>
       </c>
       <c r="AX12" t="inlineStr">
@@ -3481,17 +3481,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Le ballon sous la visière, dans le sac ! Nina refuse de creuser plus fort. Elle suit le grain de sel, jusqu'au bouton de bois. La casquette accueille le ballon, puis rentre. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. La visière a fait un nid ! Le trou a failli tout garder. La visière garde un voile de sable. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>Le ballon sous la visière, dans le sac ! Nina refuse de creuser plus fort. Nina retrouve le grain, collé au bois. La casquette accueille le ballon, puis rentre. Le bouton de bois pince le grain, et tient. Le grain a parlé, comme une lanterne. La visière a fait un nid ! Le trou a failli tout garder. La visière garde un voile de sable. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le ballon sous la visière, dans le sac ! Nina refuse de creuser plus fort. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. La casquette accueille le ballon, puis rentre. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. La visière a fait un nid ! Le trou a failli tout garder. La visière garde un voile de sable. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le ballon sous la visière, dans le sac ! Nina refuse de creuser plus fort. Nina retrouve le grain, collé au bois. La casquette accueille le ballon, puis rentre. Le bouton de bois pince le grain, et tient. Le grain a parlé, comme une lanterne. La visière a fait un nid ! Le trou a failli tout garder. La visière garde un voile de sable. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Le ballon sous la visière, dans le sac ! Nina refuse de creuser plus fort. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. La casquette accueille le ballon, puis rentre. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. La visière a fait un nid ! Le trou a failli tout garder. La visière garde un voile de sable. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>Le ballon sous la visière, dans le sac ! Nina refuse de creuser plus fort. Nina retrouve le grain, collé au bois. La casquette accueille le ballon, puis rentre. Le bouton de bois pince le grain, et tient. Le grain a parlé, comme une lanterne. La visière a fait un nid ! Le trou a failli tout garder. La visière garde un voile de sable. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit. [pause]</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -3627,15 +3627,15 @@
         <is>
           <t>enfant-f|Le ballon sous la visière, dans le sac !
 narrateur|Nina refuse de creuser plus fort.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Nina retrouve le grain, collé au bois.
 narrateur|La casquette accueille le ballon, puis rentre.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le bouton de bois pince le grain, et tient.
 papa|Le grain a parlé, comme une lanterne.
 enfant-f|La visière a fait un nid !
 maman|Le trou a failli tout garder.
 narrateur|La visière garde un voile de sable.
-papa|Tu as vu le grain, sur le bouton ?
-enfant-f|Il était sur la vitre, à la cuisine.</t>
+papa|Tu reconnais le grain, du verre ?
+enfant-f|Il a glissé du verre, tout petit.</t>
         </is>
       </c>
       <c r="AX14" t="inlineStr">
@@ -4244,17 +4244,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Le seau vide, puis la gourde dedans, dans le sac ! Nina penche le seau, loin du sable. Elle suit le grain de sel, jusqu'au bouton de bois. La gourde se tient, fraîche, au fond du seau. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. Le seau est un nid, pas un poids ! La sangle a failli tout enterrer. Le seau tient une goutte fraîche, collée au grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>Le seau vide, puis la gourde dedans, dans le sac ! Nina penche le seau, loin du sable. Elle pose le doigt sur le grain, sans presser. La gourde se tient, fraîche, au fond du seau. Le bouton parle, contre le grain. Le grain a parlé, sur le bois. Le seau est un nid, pas un poids ! La sangle a failli tout enterrer. Le seau tient une goutte fraîche, collée au grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le seau vide, puis la gourde dedans, dans le sac ! Nina penche le seau, loin du sable. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. La gourde se tient, fraîche, au fond du seau. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. Le seau est un nid, pas un poids ! La sangle a failli tout enterrer. Le seau tient une goutte fraîche, collée au grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le seau vide, puis la gourde dedans, dans le sac ! Nina penche le seau, loin du sable. Elle pose le doigt sur le grain, sans presser. La gourde se tient, fraîche, au fond du seau. Le bouton parle, contre le grain. Le grain a parlé, sur le bois. Le seau est un nid, pas un poids ! La sangle a failli tout enterrer. Le seau tient une goutte fraîche, collée au grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Le seau vide, puis la gourde dedans, dans le sac ! Nina penche le seau, loin du sable. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. La gourde se tient, fraîche, au fond du seau. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. Le seau est un nid, pas un poids ! La sangle a failli tout enterrer. Le seau tient une goutte fraîche, collée au grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>Le seau vide, puis la gourde dedans, dans le sac ! Nina penche le seau, loin du sable. Elle pose le doigt sur le grain, sans presser. La gourde se tient, fraîche, au fond du seau. Le bouton parle, contre le grain. Le grain a parlé, sur le bois. Le seau est un nid, pas un poids ! La sangle a failli tout enterrer. Le seau tient une goutte fraîche, collée au grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -4390,9 +4390,9 @@
         <is>
           <t>enfant-f|Le seau vide, puis la gourde dedans, dans le sac !
 narrateur|Nina penche le seau, loin du sable.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Elle pose le doigt sur le grain, sans presser.
 narrateur|La gourde se tient, fraîche, au fond du seau.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le bouton parle, contre le grain.
 papa|Le grain a parlé, sur le bois.
 enfant-f|Le seau est un nid, pas un poids !
 maman|La sangle a failli tout enterrer.
@@ -4617,17 +4617,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>La pomme dans le seau, puis le seau dans le sac ! Nina vide le sable, sans tirer. Elle suit le grain de sel, jusqu'au bouton de bois. La pomme se cale, et le seau rentre, léger. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. Le goûter a un seau, maintenant ! La sangle a failli tout enterrer. Une croûte de pain sent le sable, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>La pomme dans le seau, puis le seau dans le sac ! Nina vide le sable, sans tirer. Le grain de sel montre le bouton, minuscule. La pomme se cale, et le seau rentre, léger. Le sac pèse, grain sous le bois. Le grain a parlé, très bas. Le goûter a un seau, maintenant ! La sangle a failli tout enterrer. Une croûte de pain sent le sable, sous le grain. Le grain est là, tu le sens ? Oui, c'est celui de la buée.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La pomme dans le seau, puis le seau dans le sac ! Nina vide le sable, sans tirer. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. La pomme se cale, et le seau rentre, léger. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. Le goûter a un seau, maintenant ! La sangle a failli tout enterrer. Une croûte de pain sent le sable, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La pomme dans le seau, puis le seau dans le sac ! Nina vide le sable, sans tirer. Le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt; montre le bouton, minuscule. La pomme se cale, et le seau rentre, léger. Le sac pèse, grain sous le bois. Le grain a parlé, très bas. Le goûter a un seau, maintenant ! La sangle a failli tout enterrer. Une croûte de pain sent le sable, sous le grain. Le grain est là, tu le sens ? Oui, c'est celui de la buée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>La pomme dans le seau, puis le seau dans le sac ! Nina vide le sable, sans tirer. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. La pomme se cale, et le seau rentre, léger. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. Le goûter a un seau, maintenant ! La sangle a failli tout enterrer. Une croûte de pain sent le sable, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>La pomme dans le seau, puis le seau dans le sac ! Nina vide le sable, sans tirer. Le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt; montre le bouton, minuscule. La pomme se cale, et le seau rentre, léger. Le sac pèse, grain sous le bois. Le grain a parlé, très bas. Le goûter a un seau, maintenant ! La sangle a failli tout enterrer. Une croûte de pain sent le sable, sous le grain. Le grain est là, tu le sens ? Oui, c'est celui de la buée. [pause]</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4763,15 +4763,15 @@
         <is>
           <t>enfant-f|La pomme dans le seau, puis le seau dans le sac !
 narrateur|Nina vide le sable, sans tirer.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Le grain de sel montre le bouton, minuscule.
 narrateur|La pomme se cale, et le seau rentre, léger.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le sac pèse, grain sous le bois.
 papa|Le grain a parlé, très bas.
 enfant-f|Le goûter a un seau, maintenant !
 maman|La sangle a failli tout enterrer.
 narrateur|Une croûte de pain sent le sable, sous le grain.
-papa|Tu as vu le grain, sur le bouton ?
-enfant-f|Il était sur la vitre, à la cuisine.</t>
+papa|Le grain est là, tu le sens ?
+enfant-f|Oui, c'est celui de la buée.</t>
         </is>
       </c>
       <c r="AX20" t="inlineStr">
@@ -4990,17 +4990,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>La casquette en couvercle, sur le seau, dans le sac ! Nina pose la visière, sans presser le sable. Elle suit le grain de sel, jusqu'au bouton de bois. Le seau rentre, chapeau dessus, léger. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. La visière a tenu le seau ! La sangle a failli tout enterrer. La visière sert de couvercle au seau, grain dessus. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>La casquette en couvercle, sur le seau, dans le sac ! Nina pose la visière, sans presser le sable. Elle écoute le sac, et retrouve le grain. Le seau rentre, chapeau dessus, léger. Le bouton rentre, et le grain reste. Le grain a parlé, comme une lanterne. La visière a tenu le seau ! La sangle a failli tout enterrer. La visière sert de couvercle au seau, grain dessus. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La casquette en couvercle, sur le seau, dans le sac ! Nina pose la visière, sans presser le sable. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le seau rentre, chapeau dessus, léger. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. La visière a tenu le seau ! La sangle a failli tout enterrer. La visière sert de couvercle au seau, grain dessus. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La casquette en couvercle, sur le seau, dans le sac ! Nina pose la visière, sans presser le sable. Elle écoute le sac, et retrouve le grain. Le seau rentre, chapeau dessus, léger. Le bouton rentre, et le grain reste. Le grain a parlé, comme une lanterne. La visière a tenu le seau ! La sangle a failli tout enterrer. La visière sert de couvercle au seau, grain dessus. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>La casquette en couvercle, sur le seau, dans le sac ! Nina pose la visière, sans presser le sable. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le seau rentre, chapeau dessus, léger. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. La visière a tenu le seau ! La sangle a failli tout enterrer. La visière sert de couvercle au seau, grain dessus. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>La casquette en couvercle, sur le seau, dans le sac ! Nina pose la visière, sans presser le sable. Elle écoute le sac, et retrouve le grain. Le seau rentre, chapeau dessus, léger. Le bouton rentre, et le grain reste. Le grain a parlé, comme une lanterne. La visière a tenu le seau ! La sangle a failli tout enterrer. La visière sert de couvercle au seau, grain dessus. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit. [pause]</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -5136,15 +5136,15 @@
         <is>
           <t>enfant-f|La casquette en couvercle, sur le seau, dans le sac !
 narrateur|Nina pose la visière, sans presser le sable.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Elle écoute le sac, et retrouve le grain.
 narrateur|Le seau rentre, chapeau dessus, léger.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le bouton rentre, et le grain reste.
 papa|Le grain a parlé, comme une lanterne.
 enfant-f|La visière a tenu le seau !
 maman|La sangle a failli tout enterrer.
 narrateur|La visière sert de couvercle au seau, grain dessus.
-papa|Tu as vu le grain, sur le bouton ?
-enfant-f|Il était sur la vitre, à la cuisine.</t>
+papa|Tu reconnais le grain, du verre ?
+enfant-f|Il a glissé du verre, tout petit.</t>
         </is>
       </c>
       <c r="AX22" t="inlineStr">
@@ -5753,17 +5753,17 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Le doudou dans le sac, la gourde à côté ! Nina soulève le tissu, grain après grain. Elle suit le grain de sel, jusqu'au bouton de bois. Le doudou rentre, la gourde se cale, fraîche. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. Il a un nid, plus le rebord ! Le sable a failli tout garder. L'oreille du doudou a un fil de sable, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>Le doudou dans le sac, la gourde à côté ! Nina soulève le tissu, grain après grain. Nina regarde le grain, collé au bois rêche. Le doudou rentre, la gourde se cale, fraîche. Le bois ferme, grain coincé, gentiment. Le grain a parlé, sur le bois. Il a un nid, plus le rebord ! Le sable a failli tout garder. L'oreille du doudou a un fil de sable, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le doudou dans le sac, la gourde à côté ! Nina soulève le tissu, grain après grain. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le doudou rentre, la gourde se cale, fraîche. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. Il a un nid, plus le rebord ! Le sable a failli tout garder. L'oreille du doudou a un fil de sable, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le doudou dans le sac, la gourde à côté ! Nina soulève le tissu, grain après grain. Nina regarde le grain, collé au bois rêche. Le doudou rentre, la gourde se cale, fraîche. Le bois ferme, grain coincé, gentiment. Le grain a parlé, sur le bois. Il a un nid, plus le rebord ! Le sable a failli tout garder. L'oreille du doudou a un fil de sable, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Le doudou dans le sac, la gourde à côté ! Nina soulève le tissu, grain après grain. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le doudou rentre, la gourde se cale, fraîche. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. Il a un nid, plus le rebord ! Le sable a failli tout garder. L'oreille du doudou a un fil de sable, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>Le doudou dans le sac, la gourde à côté ! Nina soulève le tissu, grain après grain. Nina regarde le grain, collé au bois rêche. Le doudou rentre, la gourde se cale, fraîche. Le bois ferme, grain coincé, gentiment. Le grain a parlé, sur le bois. Il a un nid, plus le rebord ! Le sable a failli tout garder. L'oreille du doudou a un fil de sable, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -5899,9 +5899,9 @@
         <is>
           <t>enfant-f|Le doudou dans le sac, la gourde à côté !
 narrateur|Nina soulève le tissu, grain après grain.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Nina regarde le grain, collé au bois rêche.
 narrateur|Le doudou rentre, la gourde se cale, fraîche.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le bois ferme, grain coincé, gentiment.
 papa|Le grain a parlé, sur le bois.
 enfant-f|Il a un nid, plus le rebord !
 maman|Le sable a failli tout garder.
@@ -6122,17 +6122,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>La pomme dans les bras du doudou, dans le sac ! Nina souffle le sable, sans vider le bac. Elle suit le grain de sel, jusqu'au bouton de bois. Le doudou rentre, la pomme au creux, ronde. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. Il tient le goûter, maintenant ! Le sable a failli tout garder. La pomme chauffe dans les bras du doudou. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>La pomme dans les bras du doudou, dans le sac ! Nina souffle le sable, sans vider le bac. Le grain brille, et sa main ralentit. Le doudou rentre, la pomme au creux, ronde. Le bouton tient, grain au chaud. Le grain a parlé, très bas. Il tient le goûter, maintenant ! Le sable a failli tout garder. La pomme chauffe dans les bras du doudou. Le grain est là, tu le sens ? Oui, c'est celui de la buée.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La pomme dans les bras du doudou, dans le sac ! Nina souffle le sable, sans vider le bac. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le doudou rentre, la pomme au creux, ronde. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. Il tient le goûter, maintenant ! Le sable a failli tout garder. La pomme chauffe dans les bras du doudou. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La pomme dans les bras du doudou, dans le sac ! Nina souffle le sable, sans vider le bac. Le grain brille, et sa main ralentit. Le doudou rentre, la pomme au creux, ronde. Le bouton tient, grain au chaud. Le grain a parlé, très bas. Il tient le goûter, maintenant ! Le sable a failli tout garder. La pomme chauffe dans les bras du doudou. Le grain est là, tu le sens ? Oui, c'est celui de la buée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>La pomme dans les bras du doudou, dans le sac ! Nina souffle le sable, sans vider le bac. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le doudou rentre, la pomme au creux, ronde. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. Il tient le goûter, maintenant ! Le sable a failli tout garder. La pomme chauffe dans les bras du doudou. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>La pomme dans les bras du doudou, dans le sac ! Nina souffle le sable, sans vider le bac. Le grain brille, et sa main ralentit. Le doudou rentre, la pomme au creux, ronde. Le bouton tient, grain au chaud. Le grain a parlé, très bas. Il tient le goûter, maintenant ! Le sable a failli tout garder. La pomme chauffe dans les bras du doudou. Le grain est là, tu le sens ? Oui, c'est celui de la buée. [pause]</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -6268,15 +6268,15 @@
         <is>
           <t>enfant-f|La pomme dans les bras du doudou, dans le sac !
 narrateur|Nina souffle le sable, sans vider le bac.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Le grain brille, et sa main ralentit.
 narrateur|Le doudou rentre, la pomme au creux, ronde.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le bouton tient, grain au chaud.
 papa|Le grain a parlé, très bas.
 enfant-f|Il tient le goûter, maintenant !
 maman|Le sable a failli tout garder.
 narrateur|La pomme chauffe dans les bras du doudou.
-papa|Tu as vu le grain, sur le bouton ?
-enfant-f|Il était sur la vitre, à la cuisine.</t>
+papa|Le grain est là, tu le sens ?
+enfant-f|Oui, c'est celui de la buée.</t>
         </is>
       </c>
       <c r="AX28" t="inlineStr">
@@ -6491,17 +6491,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>La casquette sur le doudou, puis dans le sac ! Nina refuse de tout vider d'un coup. Elle suit le grain de sel, jusqu'au bouton de bois. Le doudou rentre, casquette sur l'oreille. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. Il a un chapeau, et un nid ! Le sable a failli tout garder. Le doudou porte la casquette, grain sur la visière. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>La casquette sur le doudou, puis dans le sac ! Nina refuse de tout vider d'un coup. Elle cherche le grain, du doigt, sur le bois. Le doudou rentre, casquette sur l'oreille. Le sac se cale, grain vers le tissu. Le grain a parlé, comme une lanterne. Il a un chapeau, et un nid ! Le sable a failli tout garder. Le doudou porte la casquette, grain sur la visière. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La casquette sur le doudou, puis dans le sac ! Nina refuse de tout vider d'un coup. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le doudou rentre, casquette sur l'oreille. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. Il a un chapeau, et un nid ! Le sable a failli tout garder. Le doudou porte la casquette, grain sur la visière. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La casquette sur le doudou, puis dans le sac ! Nina refuse de tout vider d'un coup. Elle cherche le grain, du doigt, sur le bois. Le doudou rentre, casquette sur l'oreille. Le sac se cale, grain vers le tissu. Le grain a parlé, comme une lanterne. Il a un chapeau, et un nid ! Le sable a failli tout garder. Le doudou porte la casquette, grain sur la visière. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>La casquette sur le doudou, puis dans le sac ! Nina refuse de tout vider d'un coup. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le doudou rentre, casquette sur l'oreille. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. Il a un chapeau, et un nid ! Le sable a failli tout garder. Le doudou porte la casquette, grain sur la visière. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>La casquette sur le doudou, puis dans le sac ! Nina refuse de tout vider d'un coup. Elle cherche le grain, du doigt, sur le bois. Le doudou rentre, casquette sur l'oreille. Le sac se cale, grain vers le tissu. Le grain a parlé, comme une lanterne. Il a un chapeau, et un nid ! Le sable a failli tout garder. Le doudou porte la casquette, grain sur la visière. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit. [pause]</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6637,15 +6637,15 @@
         <is>
           <t>enfant-f|La casquette sur le doudou, puis dans le sac !
 narrateur|Nina refuse de tout vider d'un coup.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Elle cherche le grain, du doigt, sur le bois.
 narrateur|Le doudou rentre, casquette sur l'oreille.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le sac se cale, grain vers le tissu.
 papa|Le grain a parlé, comme une lanterne.
 enfant-f|Il a un chapeau, et un nid !
 maman|Le sable a failli tout garder.
 narrateur|Le doudou porte la casquette, grain sur la visière.
-papa|Tu as vu le grain, sur le bouton ?
-enfant-f|Il était sur la vitre, à la cuisine.</t>
+papa|Tu reconnais le grain, du verre ?
+enfant-f|Il a glissé du verre, tout petit.</t>
         </is>
       </c>
       <c r="AX30" t="inlineStr">
@@ -8009,17 +8009,17 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Le ballon dans le sac, la gourde pour le caler ! Nina se penche sous la rampe, sans se faufiler. Elle suit le grain de sel, jusqu'au bouton de bois. Le ballon rentre, la gourde le cale, tiède. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. La gourde a tenu le ballon ! Le dessous a failli tout garder. La gourde est tiède, comme la rampe, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>Le ballon dans le sac, la gourde pour le caler ! Nina se penche sous la rampe, sans se faufiler. Nina aligne le grain, face à la rampe. Le ballon rentre, la gourde le cale, tiède. Le bouton ferme, tiède, sur le grain. Le grain a parlé, sur le bois. La gourde a tenu le ballon ! Le dessous a failli tout garder. La gourde est tiède, comme la rampe, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le ballon dans le sac, la gourde pour le caler ! Nina se penche sous la rampe, sans se faufiler. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le ballon rentre, la gourde le cale, tiède. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. La gourde a tenu le ballon ! Le dessous a failli tout garder. La gourde est tiède, comme la rampe, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le ballon dans le sac, la gourde pour le caler ! Nina se penche sous la rampe, sans se faufiler. Nina aligne le grain, face à la rampe. Le ballon rentre, la gourde le cale, tiède. Le bouton ferme, tiède, sur le grain. Le grain a parlé, sur le bois. La gourde a tenu le ballon ! Le dessous a failli tout garder. La gourde est tiède, comme la rampe, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Le ballon dans le sac, la gourde pour le caler ! Nina se penche sous la rampe, sans se faufiler. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le ballon rentre, la gourde le cale, tiède. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. La gourde a tenu le ballon ! Le dessous a failli tout garder. La gourde est tiède, comme la rampe, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>Le ballon dans le sac, la gourde pour le caler ! Nina se penche sous la rampe, sans se faufiler. Nina aligne le grain, face à la rampe. Le ballon rentre, la gourde le cale, tiède. Le bouton ferme, tiède, sur le grain. Le grain a parlé, sur le bois. La gourde a tenu le ballon ! Le dessous a failli tout garder. La gourde est tiède, comme la rampe, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -8155,9 +8155,9 @@
         <is>
           <t>enfant-f|Le ballon dans le sac, la gourde pour le caler !
 narrateur|Nina se penche sous la rampe, sans se faufiler.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Nina aligne le grain, face à la rampe.
 narrateur|Le ballon rentre, la gourde le cale, tiède.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le bouton ferme, tiède, sur le grain.
 papa|Le grain a parlé, sur le bois.
 enfant-f|La gourde a tenu le ballon !
 maman|Le dessous a failli tout garder.
@@ -8382,17 +8382,17 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Le ballon dans le sac, la pomme pour le peser ! Nina tend le bras, sans ramper. Elle suit le grain de sel, jusqu'au bouton de bois. Le ballon rentre, la pomme pèse, ronde. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. La pomme a tenu le ballon ! Le dessous a failli tout garder. La pomme a un trait lisse, collé au grain de sel. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>Le ballon dans le sac, la pomme pour le peser ! Nina tend le bras, sans ramper. Le grain de sel attend, sur le bouton de bois. Le ballon rentre, la pomme pèse, ronde. Le sac se ferme, grain contre la pomme. Le grain a parlé, très bas. La pomme a tenu le ballon ! Le dessous a failli tout garder. La pomme a un trait lisse, collé au grain de sel. Le grain est là, tu le sens ? Oui, c'est celui de la buée.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le ballon dans le sac, la pomme pour le peser ! Nina tend le bras, sans ramper. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le ballon rentre, la pomme pèse, ronde. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. La pomme a tenu le ballon ! Le dessous a failli tout garder. La pomme a un trait lisse, collé au grain de sel. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le ballon dans le sac, la pomme pour le peser ! Nina tend le bras, sans ramper. Le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt; attend, sur le bouton de bois. Le ballon rentre, la pomme pèse, ronde. Le sac se ferme, grain contre la pomme. Le grain a parlé, très bas. La pomme a tenu le ballon ! Le dessous a failli tout garder. La pomme a un trait lisse, collé au grain de sel. Le grain est là, tu le sens ? Oui, c'est celui de la buée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Le ballon dans le sac, la pomme pour le peser ! Nina tend le bras, sans ramper. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le ballon rentre, la pomme pèse, ronde. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. La pomme a tenu le ballon ! Le dessous a failli tout garder. La pomme a un trait lisse, collé au grain de sel. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>Le ballon dans le sac, la pomme pour le peser ! Nina tend le bras, sans ramper. Le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt; attend, sur le bouton de bois. Le ballon rentre, la pomme pèse, ronde. Le sac se ferme, grain contre la pomme. Le grain a parlé, très bas. La pomme a tenu le ballon ! Le dessous a failli tout garder. La pomme a un trait lisse, collé au grain de sel. Le grain est là, tu le sens ? Oui, c'est celui de la buée. [pause]</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -8528,15 +8528,15 @@
         <is>
           <t>enfant-f|Le ballon dans le sac, la pomme pour le peser !
 narrateur|Nina tend le bras, sans ramper.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Le grain de sel attend, sur le bouton de bois.
 narrateur|Le ballon rentre, la pomme pèse, ronde.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le sac se ferme, grain contre la pomme.
 papa|Le grain a parlé, très bas.
 enfant-f|La pomme a tenu le ballon !
 maman|Le dessous a failli tout garder.
 narrateur|La pomme a un trait lisse, collé au grain de sel.
-papa|Tu as vu le grain, sur le bouton ?
-enfant-f|Il était sur la vitre, à la cuisine.</t>
+papa|Le grain est là, tu le sens ?
+enfant-f|Oui, c'est celui de la buée.</t>
         </is>
       </c>
       <c r="AX40" t="inlineStr">
@@ -8755,17 +8755,17 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>La casquette comme un filet, pour le ballon ! Nina glisse la visière sous la rampe, lentement. Elle suit le grain de sel, jusqu'au bouton de bois. Le ballon roule dans la visière, puis dans le sac. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. La visière a attrapé, sans foncer ! Le dessous a failli tout garder. La visière tient une poussière de rampe, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>La casquette comme un filet, pour le ballon ! Nina glisse la visière sous la rampe, lentement. Elle touche le grain, puis le bouton. Le ballon roule dans la visière, puis dans le sac. Le bouton de bois serre le grain, sans pincer. Le grain a parlé, comme une lanterne. La visière a attrapé, sans foncer ! Le dessous a failli tout garder. La visière tient une poussière de rampe, près du grain. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La casquette comme un filet, pour le ballon ! Nina glisse la visière sous la rampe, lentement. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le ballon roule dans la visière, puis dans le sac. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. La visière a attrapé, sans foncer ! Le dessous a failli tout garder. La visière tient une poussière de rampe, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La casquette comme un filet, pour le ballon ! Nina glisse la visière sous la rampe, lentement. Elle touche le grain, puis le bouton. Le ballon roule dans la visière, puis dans le sac. Le bouton de bois serre le grain, sans pincer. Le grain a parlé, comme une lanterne. La visière a attrapé, sans foncer ! Le dessous a failli tout garder. La visière tient une poussière de rampe, près du grain. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>La casquette comme un filet, pour le ballon ! Nina glisse la visière sous la rampe, lentement. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le ballon roule dans la visière, puis dans le sac. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. La visière a attrapé, sans foncer ! Le dessous a failli tout garder. La visière tient une poussière de rampe, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>La casquette comme un filet, pour le ballon ! Nina glisse la visière sous la rampe, lentement. Elle touche le grain, puis le bouton. Le ballon roule dans la visière, puis dans le sac. Le bouton de bois serre le grain, sans pincer. Le grain a parlé, comme une lanterne. La visière a attrapé, sans foncer ! Le dessous a failli tout garder. La visière tient une poussière de rampe, près du grain. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit. [pause]</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -8901,15 +8901,15 @@
         <is>
           <t>enfant-f|La casquette comme un filet, pour le ballon !
 narrateur|Nina glisse la visière sous la rampe, lentement.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Elle touche le grain, puis le bouton.
 narrateur|Le ballon roule dans la visière, puis dans le sac.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le bouton de bois serre le grain, sans pincer.
 papa|Le grain a parlé, comme une lanterne.
 enfant-f|La visière a attrapé, sans foncer !
 maman|Le dessous a failli tout garder.
 narrateur|La visière tient une poussière de rampe, près du grain.
-papa|Tu as vu le grain, sur le bouton ?
-enfant-f|Il était sur la vitre, à la cuisine.</t>
+papa|Tu reconnais le grain, du verre ?
+enfant-f|Il a glissé du verre, tout petit.</t>
         </is>
       </c>
       <c r="AX42" t="inlineStr">
@@ -9514,17 +9514,17 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Le seau en bas, la gourde pour l'accueillir ! Nina descend, une marche après l'autre. Elle suit le grain de sel, jusqu'au bouton de bois. Le seau rentre, la gourde au fond, fraîche. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. Le seau a un nid, plus la pente ! La rampe a failli tout garder. Le seau garde une goutte de rampe, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>Le seau en bas, la gourde pour l'accueillir ! Nina descend, une marche après l'autre. Nina suit le grain, du pied au bois. Le seau rentre, la gourde au fond, fraîche. Le bouton parle, au pied de la rampe. Le grain a parlé, sur le bois. Le seau a un nid, plus la pente ! La rampe a failli tout garder. Le seau garde une goutte de rampe, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le seau en bas, la gourde pour l'accueillir ! Nina descend, une marche après l'autre. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le seau rentre, la gourde au fond, fraîche. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. Le seau a un nid, plus la pente ! La rampe a failli tout garder. Le seau garde une goutte de rampe, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le seau en bas, la gourde pour l'accueillir ! Nina descend, une marche après l'autre. Nina suit le grain, du pied au bois. Le seau rentre, la gourde au fond, fraîche. Le bouton parle, au pied de la rampe. Le grain a parlé, sur le bois. Le seau a un nid, plus la pente ! La rampe a failli tout garder. Le seau garde une goutte de rampe, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Le seau en bas, la gourde pour l'accueillir ! Nina descend, une marche après l'autre. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le seau rentre, la gourde au fond, fraîche. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. Le seau a un nid, plus la pente ! La rampe a failli tout garder. Le seau garde une goutte de rampe, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>Le seau en bas, la gourde pour l'accueillir ! Nina descend, une marche après l'autre. Nina suit le grain, du pied au bois. Le seau rentre, la gourde au fond, fraîche. Le bouton parle, au pied de la rampe. Le grain a parlé, sur le bois. Le seau a un nid, plus la pente ! La rampe a failli tout garder. Le seau garde une goutte de rampe, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -9660,9 +9660,9 @@
         <is>
           <t>enfant-f|Le seau en bas, la gourde pour l'accueillir !
 narrateur|Nina descend, une marche après l'autre.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Nina suit le grain, du pied au bois.
 narrateur|Le seau rentre, la gourde au fond, fraîche.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le bouton parle, au pied de la rampe.
 papa|Le grain a parlé, sur le bois.
 enfant-f|Le seau a un nid, plus la pente !
 maman|La rampe a failli tout garder.
@@ -9887,17 +9887,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>La pomme dans le seau, après la rampe ! Nina attend que le seau se taise. Elle suit le grain de sel, jusqu'au bouton de bois. La pomme se cale, le seau rentre, tiède. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. Le goûter a voyagé, sans glisser ! La rampe a failli tout garder. Une croûte tiède sent le plastique, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>La pomme dans le seau, après la rampe ! Nina attend que le seau se taise. Le grain de sel tremble, et elle s'arrête. La pomme se cale, le seau rentre, tiède. Le sac pèse, grain sous la croûte. Le grain a parlé, très bas. Le goûter a voyagé, sans glisser ! La rampe a failli tout garder. Une croûte tiède sent le plastique, près du grain. Le grain est là, tu le sens ? Oui, c'est celui de la buée.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La pomme dans le seau, après la rampe ! Nina attend que le seau se taise. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. La pomme se cale, le seau rentre, tiède. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. Le goûter a voyagé, sans glisser ! La rampe a failli tout garder. Une croûte tiède sent le plastique, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La pomme dans le seau, après la rampe ! Nina attend que le seau se taise. Le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt; tremble, et elle s'arrête. La pomme se cale, le seau rentre, tiède. Le sac pèse, grain sous la croûte. Le grain a parlé, très bas. Le goûter a voyagé, sans glisser ! La rampe a failli tout garder. Une croûte tiède sent le plastique, près du grain. Le grain est là, tu le sens ? Oui, c'est celui de la buée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>La pomme dans le seau, après la rampe ! Nina attend que le seau se taise. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. La pomme se cale, le seau rentre, tiède. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. Le goûter a voyagé, sans glisser ! La rampe a failli tout garder. Une croûte tiède sent le plastique, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>La pomme dans le seau, après la rampe ! Nina attend que le seau se taise. Le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt; tremble, et elle s'arrête. La pomme se cale, le seau rentre, tiède. Le sac pèse, grain sous la croûte. Le grain a parlé, très bas. Le goûter a voyagé, sans glisser ! La rampe a failli tout garder. Une croûte tiède sent le plastique, près du grain. Le grain est là, tu le sens ? Oui, c'est celui de la buée. [pause]</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -10033,15 +10033,15 @@
         <is>
           <t>enfant-f|La pomme dans le seau, après la rampe !
 narrateur|Nina attend que le seau se taise.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Le grain de sel tremble, et elle s'arrête.
 narrateur|La pomme se cale, le seau rentre, tiède.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le sac pèse, grain sous la croûte.
 papa|Le grain a parlé, très bas.
 enfant-f|Le goûter a voyagé, sans glisser !
 maman|La rampe a failli tout garder.
 narrateur|Une croûte tiède sent le plastique, près du grain.
-papa|Tu as vu le grain, sur le bouton ?
-enfant-f|Il était sur la vitre, à la cuisine.</t>
+papa|Le grain est là, tu le sens ?
+enfant-f|Oui, c'est celui de la buée.</t>
         </is>
       </c>
       <c r="AX48" t="inlineStr">
@@ -10260,17 +10260,17 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>La casquette dans le seau, puis le seau dans le sac ! Nina refuse de relancer le seau. Elle suit le grain de sel, jusqu'au bouton de bois. La visière se cale, le seau rentre, léger. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. La visière a voyagé, sans voile ! La rampe a failli tout garder. La visière a voyagé dans le seau, grain au bord. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>La casquette dans le seau, puis le seau dans le sac ! Nina refuse de relancer le seau. Elle retrouve le grain, au milieu du bouton. La visière se cale, le seau rentre, léger. Le bouton rentre, visière au bord. Le grain a parlé, comme une lanterne. La visière a voyagé, sans voile ! La rampe a failli tout garder. La visière a voyagé dans le seau, grain au bord. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La casquette dans le seau, puis le seau dans le sac ! Nina refuse de relancer le seau. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. La visière se cale, le seau rentre, léger. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. La visière a voyagé, sans voile ! La rampe a failli tout garder. La visière a voyagé dans le seau, grain au bord. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La casquette dans le seau, puis le seau dans le sac ! Nina refuse de relancer le seau. Elle retrouve le grain, au milieu du bouton. La visière se cale, le seau rentre, léger. Le bouton rentre, visière au bord. Le grain a parlé, comme une lanterne. La visière a voyagé, sans voile ! La rampe a failli tout garder. La visière a voyagé dans le seau, grain au bord. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>La casquette dans le seau, puis le seau dans le sac ! Nina refuse de relancer le seau. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. La visière se cale, le seau rentre, léger. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. La visière a voyagé, sans voile ! La rampe a failli tout garder. La visière a voyagé dans le seau, grain au bord. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>La casquette dans le seau, puis le seau dans le sac ! Nina refuse de relancer le seau. Elle retrouve le grain, au milieu du bouton. La visière se cale, le seau rentre, léger. Le bouton rentre, visière au bord. Le grain a parlé, comme une lanterne. La visière a voyagé, sans voile ! La rampe a failli tout garder. La visière a voyagé dans le seau, grain au bord. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit. [pause]</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -10406,15 +10406,15 @@
         <is>
           <t>enfant-f|La casquette dans le seau, puis le seau dans le sac !
 narrateur|Nina refuse de relancer le seau.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Elle retrouve le grain, au milieu du bouton.
 narrateur|La visière se cale, le seau rentre, léger.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le bouton rentre, visière au bord.
 papa|Le grain a parlé, comme une lanterne.
 enfant-f|La visière a voyagé, sans voile !
 maman|La rampe a failli tout garder.
 narrateur|La visière a voyagé dans le seau, grain au bord.
-papa|Tu as vu le grain, sur le bouton ?
-enfant-f|Il était sur la vitre, à la cuisine.</t>
+papa|Tu reconnais le grain, du verre ?
+enfant-f|Il a glissé du verre, tout petit.</t>
         </is>
       </c>
       <c r="AX50" t="inlineStr">
@@ -11023,17 +11023,17 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Le doudou dans le sac, la gourde contre l'oreille ! Nina pose le tissu, sans le lancer. Elle suit le grain de sel, jusqu'au bouton de bois. Le doudou rentre, la gourde le cale, tiède. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. Il a un nid, plus le vent ! La rampe a failli l'emporter. Le doudou sent la rampe, grain de sel dans un pli. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>Le doudou dans le sac, la gourde contre l'oreille ! Nina pose le tissu, sans le lancer. Nina pose l'oreille près du sac, et voit le grain. Le doudou rentre, la gourde le cale, tiède. Le bois ferme, grain dans un pli. Le grain a parlé, sur le bois. Il a un nid, plus le vent ! La rampe a failli l'emporter. Le doudou sent la rampe, grain de sel dans un pli. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le doudou dans le sac, la gourde contre l'oreille ! Nina pose le tissu, sans le lancer. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le doudou rentre, la gourde le cale, tiède. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. Il a un nid, plus le vent ! La rampe a failli l'emporter. Le doudou sent la rampe, grain de sel dans un pli. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le doudou dans le sac, la gourde contre l'oreille ! Nina pose le tissu, sans le lancer. Nina pose l'oreille près du sac, et voit le grain. Le doudou rentre, la gourde le cale, tiède. Le bois ferme, grain dans un pli. Le grain a parlé, sur le bois. Il a un nid, plus le vent ! La rampe a failli l'emporter. Le doudou sent la rampe, &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt; dans un pli. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Le doudou dans le sac, la gourde contre l'oreille ! Nina pose le tissu, sans le lancer. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le doudou rentre, la gourde le cale, tiède. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. Il a un nid, plus le vent ! La rampe a failli l'emporter. Le doudou sent la rampe, grain de sel dans un pli. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>Le doudou dans le sac, la gourde contre l'oreille ! Nina pose le tissu, sans le lancer. Nina pose l'oreille près du sac, et voit le grain. Le doudou rentre, la gourde le cale, tiède. Le bois ferme, grain dans un pli. Le grain a parlé, sur le bois. Il a un nid, plus le vent ! La rampe a failli l'emporter. Le doudou sent la rampe, &lt;emphasis&gt;grain de sel&lt;/emphasis&gt; dans un pli. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -11169,9 +11169,9 @@
         <is>
           <t>enfant-f|Le doudou dans le sac, la gourde contre l'oreille !
 narrateur|Nina pose le tissu, sans le lancer.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Nina pose l'oreille près du sac, et voit le grain.
 narrateur|Le doudou rentre, la gourde le cale, tiède.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le bois ferme, grain dans un pli.
 papa|Le grain a parlé, sur le bois.
 enfant-f|Il a un nid, plus le vent !
 maman|La rampe a failli l'emporter.
@@ -11396,17 +11396,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>La pomme pour le doudou, dans le sac ! Nina serre moins fort, et avance. Elle suit le grain de sel, jusqu'au bouton de bois. Le doudou rentre, la pomme au creux, ronde. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. Il tient le goûter, sans le vent ! La rampe a failli l'emporter. La pomme sent le tissu du doudou, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>La pomme pour le doudou, dans le sac ! Nina serre moins fort, et avance. Le grain de sel luit, contre le bois rêche. Le doudou rentre, la pomme au creux, ronde. Le bouton tient, grain contre la pomme. Le grain a parlé, très bas. Il tient le goûter, sans le vent ! La rampe a failli l'emporter. La pomme sent le tissu du doudou, sous le grain. Le grain est là, tu le sens ? Oui, c'est celui de la buée.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La pomme pour le doudou, dans le sac ! Nina serre moins fort, et avance. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le doudou rentre, la pomme au creux, ronde. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. Il tient le goûter, sans le vent ! La rampe a failli l'emporter. La pomme sent le tissu du doudou, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La pomme pour le doudou, dans le sac ! Nina serre moins fort, et avance. Le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt; luit, contre le bois rêche. Le doudou rentre, la pomme au creux, ronde. Le bouton tient, grain contre la pomme. Le grain a parlé, très bas. Il tient le goûter, sans le vent ! La rampe a failli l'emporter. La pomme sent le tissu du doudou, sous le grain. Le grain est là, tu le sens ? Oui, c'est celui de la buée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>La pomme pour le doudou, dans le sac ! Nina serre moins fort, et avance. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le doudou rentre, la pomme au creux, ronde. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. Il tient le goûter, sans le vent ! La rampe a failli l'emporter. La pomme sent le tissu du doudou, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>La pomme pour le doudou, dans le sac ! Nina serre moins fort, et avance. Le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt; luit, contre le bois rêche. Le doudou rentre, la pomme au creux, ronde. Le bouton tient, grain contre la pomme. Le grain a parlé, très bas. Il tient le goûter, sans le vent ! La rampe a failli l'emporter. La pomme sent le tissu du doudou, sous le grain. Le grain est là, tu le sens ? Oui, c'est celui de la buée. [pause]</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -11542,15 +11542,15 @@
         <is>
           <t>enfant-f|La pomme pour le doudou, dans le sac !
 narrateur|Nina serre moins fort, et avance.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Le grain de sel luit, contre le bois rêche.
 narrateur|Le doudou rentre, la pomme au creux, ronde.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le bouton tient, grain contre la pomme.
 papa|Le grain a parlé, très bas.
 enfant-f|Il tient le goûter, sans le vent !
 maman|La rampe a failli l'emporter.
 narrateur|La pomme sent le tissu du doudou, sous le grain.
-papa|Tu as vu le grain, sur le bouton ?
-enfant-f|Il était sur la vitre, à la cuisine.</t>
+papa|Le grain est là, tu le sens ?
+enfant-f|Oui, c'est celui de la buée.</t>
         </is>
       </c>
       <c r="AX56" t="inlineStr">
@@ -11769,17 +11769,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>La casquette sur le doudou, avant le sac ! Nina pose la visière, oreille à l'abri. Elle suit le grain de sel, jusqu'au bouton de bois. Le doudou rentre, casquette contre le vent. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. Il a un chapeau, et un nid ! La rampe a failli l'emporter. Un poil de doudou colle à la visière, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>La casquette sur le doudou, avant le sac ! Nina pose la visière, oreille à l'abri. Elle garde le grain, sous l'ongle, une seconde. Le doudou rentre, casquette contre le vent. Le sac se cale, grain sous la visière. Le grain a parlé, comme une lanterne. Il a un chapeau, et un nid ! La rampe a failli l'emporter. Un poil de doudou colle à la visière, près du grain. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La casquette sur le doudou, avant le sac ! Nina pose la visière, oreille à l'abri. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le doudou rentre, casquette contre le vent. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. Il a un chapeau, et un nid ! La rampe a failli l'emporter. Un poil de doudou colle à la visière, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La casquette sur le doudou, avant le sac ! Nina pose la visière, oreille à l'abri. Elle garde le grain, sous l'ongle, une seconde. Le doudou rentre, casquette contre le vent. Le sac se cale, grain sous la visière. Le grain a parlé, comme une lanterne. Il a un chapeau, et un nid ! La rampe a failli l'emporter. Un poil de doudou colle à la visière, près du grain. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>La casquette sur le doudou, avant le sac ! Nina pose la visière, oreille à l'abri. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le doudou rentre, casquette contre le vent. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. Il a un chapeau, et un nid ! La rampe a failli l'emporter. Un poil de doudou colle à la visière, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>La casquette sur le doudou, avant le sac ! Nina pose la visière, oreille à l'abri. Elle garde le grain, sous l'ongle, une seconde. Le doudou rentre, casquette contre le vent. Le sac se cale, grain sous la visière. Le grain a parlé, comme une lanterne. Il a un chapeau, et un nid ! La rampe a failli l'emporter. Un poil de doudou colle à la visière, près du grain. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit. [pause]</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -11915,15 +11915,15 @@
         <is>
           <t>enfant-f|La casquette sur le doudou, avant le sac !
 narrateur|Nina pose la visière, oreille à l'abri.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Elle garde le grain, sous l'ongle, une seconde.
 narrateur|Le doudou rentre, casquette contre le vent.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le sac se cale, grain sous la visière.
 papa|Le grain a parlé, comme une lanterne.
 enfant-f|Il a un chapeau, et un nid !
 maman|La rampe a failli l'emporter.
 narrateur|Un poil de doudou colle à la visière, près du grain.
-papa|Tu as vu le grain, sur le bouton ?
-enfant-f|Il était sur la vitre, à la cuisine.</t>
+papa|Tu reconnais le grain, du verre ?
+enfant-f|Il a glissé du verre, tout petit.</t>
         </is>
       </c>
       <c r="AX58" t="inlineStr">
@@ -13283,17 +13283,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Le ballon dans le sac, la gourde pour le nid ! Nina contourne le siège, sans ramper. Elle suit le grain de sel, jusqu'au bouton de bois. Le ballon rentre, la gourde le cale, fraîche. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. La gourde a fait le nid ! L'ombre a failli tout garder. La gourde a une marque d'herbe, sous le grain de sel. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>Le ballon dans le sac, la gourde pour le nid ! Nina contourne le siège, sans ramper. Nina contourne le grain, puis le bouton. Le ballon rentre, la gourde le cale, fraîche. Le bouton ferme, frais, sur le grain. Le grain a parlé, sur le bois. La gourde a fait le nid ! L'ombre a failli tout garder. La gourde a une marque d'herbe, sous le grain de sel. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le ballon dans le sac, la gourde pour le nid ! Nina contourne le siège, sans ramper. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le ballon rentre, la gourde le cale, fraîche. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. La gourde a fait le nid ! L'ombre a failli tout garder. La gourde a une marque d'herbe, sous le grain de sel. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le ballon dans le sac, la gourde pour le nid ! Nina contourne le siège, sans ramper. Nina contourne le grain, puis le bouton. Le ballon rentre, la gourde le cale, fraîche. Le bouton ferme, frais, sur le grain. Le grain a parlé, sur le bois. La gourde a fait le nid ! L'ombre a failli tout garder. La gourde a une marque d'herbe, sous le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Le ballon dans le sac, la gourde pour le nid ! Nina contourne le siège, sans ramper. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le ballon rentre, la gourde le cale, fraîche. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. La gourde a fait le nid ! L'ombre a failli tout garder. La gourde a une marque d'herbe, sous le grain de sel. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>Le ballon dans le sac, la gourde pour le nid ! Nina contourne le siège, sans ramper. Nina contourne le grain, puis le bouton. Le ballon rentre, la gourde le cale, fraîche. Le bouton ferme, frais, sur le grain. Le grain a parlé, sur le bois. La gourde a fait le nid ! L'ombre a failli tout garder. La gourde a une marque d'herbe, sous le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -13429,9 +13429,9 @@
         <is>
           <t>enfant-f|Le ballon dans le sac, la gourde pour le nid !
 narrateur|Nina contourne le siège, sans ramper.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Nina contourne le grain, puis le bouton.
 narrateur|Le ballon rentre, la gourde le cale, fraîche.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le bouton ferme, frais, sur le grain.
 papa|Le grain a parlé, sur le bois.
 enfant-f|La gourde a fait le nid !
 maman|L'ombre a failli tout garder.
@@ -13656,17 +13656,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>La pomme comme un siège, pour le ballon, dans le sac ! Nina tend le bras derrière, sans se coucher. Elle suit le grain de sel, jusqu'au bouton de bois. Le ballon rentre, la pomme le cale, froide. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. La pomme a tenu le ballon ! L'ombre a failli tout garder. La pomme est froide, comme la chaîne, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>La pomme comme un siège, pour le ballon, dans le sac ! Nina tend le bras derrière, sans se coucher. Le grain de sel pique, comme à la vitre. Le ballon rentre, la pomme le cale, froide. Le sac se ferme, grain contre la chaîne. Le grain a parlé, très bas. La pomme a tenu le ballon ! L'ombre a failli tout garder. La pomme est froide, comme la chaîne, près du grain. Le grain est là, tu le sens ? Oui, c'est celui de la buée.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La pomme comme un siège, pour le ballon, dans le sac ! Nina tend le bras derrière, sans se coucher. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le ballon rentre, la pomme le cale, froide. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. La pomme a tenu le ballon ! L'ombre a failli tout garder. La pomme est froide, comme la chaîne, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La pomme comme un siège, pour le ballon, dans le sac ! Nina tend le bras derrière, sans se coucher. Le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt; pique, comme à la vitre. Le ballon rentre, la pomme le cale, froide. Le sac se ferme, grain contre la chaîne. Le grain a parlé, très bas. La pomme a tenu le ballon ! L'ombre a failli tout garder. La pomme est froide, comme la chaîne, près du grain. Le grain est là, tu le sens ? Oui, c'est celui de la buée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>La pomme comme un siège, pour le ballon, dans le sac ! Nina tend le bras derrière, sans se coucher. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le ballon rentre, la pomme le cale, froide. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. La pomme a tenu le ballon ! L'ombre a failli tout garder. La pomme est froide, comme la chaîne, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>La pomme comme un siège, pour le ballon, dans le sac ! Nina tend le bras derrière, sans se coucher. Le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt; pique, comme à la vitre. Le ballon rentre, la pomme le cale, froide. Le sac se ferme, grain contre la chaîne. Le grain a parlé, très bas. La pomme a tenu le ballon ! L'ombre a failli tout garder. La pomme est froide, comme la chaîne, près du grain. Le grain est là, tu le sens ? Oui, c'est celui de la buée. [pause]</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -13802,15 +13802,15 @@
         <is>
           <t>enfant-f|La pomme comme un siège, pour le ballon, dans le sac !
 narrateur|Nina tend le bras derrière, sans se coucher.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Le grain de sel pique, comme à la vitre.
 narrateur|Le ballon rentre, la pomme le cale, froide.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le sac se ferme, grain contre la chaîne.
 papa|Le grain a parlé, très bas.
 enfant-f|La pomme a tenu le ballon !
 maman|L'ombre a failli tout garder.
 narrateur|La pomme est froide, comme la chaîne, près du grain.
-papa|Tu as vu le grain, sur le bouton ?
-enfant-f|Il était sur la vitre, à la cuisine.</t>
+papa|Le grain est là, tu le sens ?
+enfant-f|Oui, c'est celui de la buée.</t>
         </is>
       </c>
       <c r="AX68" t="inlineStr">
@@ -14025,17 +14025,17 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>La casquette comme un hamac, pour le ballon ! Nina glisse la visière sous le siège, lentement. Elle suit le grain de sel, jusqu'au bouton de bois. Le ballon roule dans la visière, puis dans le sac. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. La visière a attrapé, sans ramper ! L'ombre a failli tout garder. La visière a un pli de chaîne, sous le grain de sel. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>La casquette comme un hamac, pour le ballon ! Nina glisse la visière sous le siège, lentement. Elle reconnaît le grain, minuscule, sur le bois. Le ballon roule dans la visière, puis dans le sac. Le bouton de bois accueille le grain, et tient. Le grain a parlé, comme une lanterne. La visière a attrapé, sans ramper ! L'ombre a failli tout garder. La visière a un pli de chaîne, sous le grain de sel. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La casquette comme un hamac, pour le ballon ! Nina glisse la visière sous le siège, lentement. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le ballon roule dans la visière, puis dans le sac. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. La visière a attrapé, sans ramper ! L'ombre a failli tout garder. La visière a un pli de chaîne, sous le grain de sel. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La casquette comme un hamac, pour le ballon ! Nina glisse la visière sous le siège, lentement. Elle reconnaît le grain, minuscule, sur le bois. Le ballon roule dans la visière, puis dans le sac. Le bouton de bois accueille le grain, et tient. Le grain a parlé, comme une lanterne. La visière a attrapé, sans ramper ! L'ombre a failli tout garder. La visière a un pli de chaîne, sous le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>La casquette comme un hamac, pour le ballon ! Nina glisse la visière sous le siège, lentement. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le ballon roule dans la visière, puis dans le sac. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. La visière a attrapé, sans ramper ! L'ombre a failli tout garder. La visière a un pli de chaîne, sous le grain de sel. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>La casquette comme un hamac, pour le ballon ! Nina glisse la visière sous le siège, lentement. Elle reconnaît le grain, minuscule, sur le bois. Le ballon roule dans la visière, puis dans le sac. Le bouton de bois accueille le grain, et tient. Le grain a parlé, comme une lanterne. La visière a attrapé, sans ramper ! L'ombre a failli tout garder. La visière a un pli de chaîne, sous le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit. [pause]</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -14171,15 +14171,15 @@
         <is>
           <t>enfant-f|La casquette comme un hamac, pour le ballon !
 narrateur|Nina glisse la visière sous le siège, lentement.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Elle reconnaît le grain, minuscule, sur le bois.
 narrateur|Le ballon roule dans la visière, puis dans le sac.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le bouton de bois accueille le grain, et tient.
 papa|Le grain a parlé, comme une lanterne.
 enfant-f|La visière a attrapé, sans ramper !
 maman|L'ombre a failli tout garder.
 narrateur|La visière a un pli de chaîne, sous le grain de sel.
-papa|Tu as vu le grain, sur le bouton ?
-enfant-f|Il était sur la vitre, à la cuisine.</t>
+papa|Tu reconnais le grain, du verre ?
+enfant-f|Il a glissé du verre, tout petit.</t>
         </is>
       </c>
       <c r="AX70" t="inlineStr">
@@ -14788,17 +14788,17 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Je décroche le seau, puis la gourde dans le sac ! Nina tourne la sangle, sans tirer. Elle suit le grain de sel, jusqu'au bouton de bois. Le seau rentre, la gourde au fond, fraîche. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. Le seau est libre, et dedans ! La chaîne a failli tout garder. Le seau sent l'herbe, grain de sel au fond. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>Je décroche le seau, puis la gourde dans le sac ! Nina tourne la sangle, sans tirer. Nina souffle sur le grain, collé au bouton. Le seau rentre, la gourde au fond, fraîche. Le bouton parle, seau libre. Le grain a parlé, sur le bois. Le seau est libre, et dedans ! La chaîne a failli tout garder. Le seau sent l'herbe, grain de sel au fond. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Je décroche le seau, puis la gourde dans le sac ! Nina tourne la sangle, sans tirer. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le seau rentre, la gourde au fond, fraîche. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. Le seau est libre, et dedans ! La chaîne a failli tout garder. Le seau sent l'herbe, grain de sel au fond. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Je décroche le seau, puis la gourde dans le sac ! Nina tourne la sangle, sans tirer. Nina souffle sur le grain, collé au bouton. Le seau rentre, la gourde au fond, fraîche. Le bouton parle, seau libre. Le grain a parlé, sur le bois. Le seau est libre, et dedans ! La chaîne a failli tout garder. Le seau sent l'herbe, &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt; au fond. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Je décroche le seau, puis la gourde dans le sac ! Nina tourne la sangle, sans tirer. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le seau rentre, la gourde au fond, fraîche. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. Le seau est libre, et dedans ! La chaîne a failli tout garder. Le seau sent l'herbe, grain de sel au fond. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>Je décroche le seau, puis la gourde dans le sac ! Nina tourne la sangle, sans tirer. Nina souffle sur le grain, collé au bouton. Le seau rentre, la gourde au fond, fraîche. Le bouton parle, seau libre. Le grain a parlé, sur le bois. Le seau est libre, et dedans ! La chaîne a failli tout garder. Le seau sent l'herbe, &lt;emphasis&gt;grain de sel&lt;/emphasis&gt; au fond. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -14934,9 +14934,9 @@
         <is>
           <t>enfant-f|Je décroche le seau, puis la gourde dans le sac !
 narrateur|Nina tourne la sangle, sans tirer.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Nina souffle sur le grain, collé au bouton.
 narrateur|Le seau rentre, la gourde au fond, fraîche.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le bouton parle, seau libre.
 papa|Le grain a parlé, sur le bois.
 enfant-f|Le seau est libre, et dedans !
 maman|La chaîne a failli tout garder.
@@ -15161,17 +15161,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>La pomme dans le seau, quand la sangle est libre ! Nina attend que la chaîne se taise. Elle suit le grain de sel, jusqu'au bouton de bois. La pomme se cale, le seau rentre, léger. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. Le goûter a un seau, sans chaîne ! La chaîne a failli tout garder. Une croûte garde l'ombre de la chaîne, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>La pomme dans le seau, quand la sangle est libre ! Nina attend que la chaîne se taise. Le grain de sel reste, malgré la chaîne. La pomme se cale, le seau rentre, léger. Le sac pèse, grain près de la croûte. Le grain a parlé, très bas. Le goûter a un seau, sans chaîne ! La chaîne a failli tout garder. Une croûte garde l'ombre de la chaîne, près du grain. Le grain est là, tu le sens ? Oui, c'est celui de la buée.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La pomme dans le seau, quand la sangle est libre ! Nina attend que la chaîne se taise. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. La pomme se cale, le seau rentre, léger. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. Le goûter a un seau, sans chaîne ! La chaîne a failli tout garder. Une croûte garde l'ombre de la chaîne, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La pomme dans le seau, quand la sangle est libre ! Nina attend que la chaîne se taise. Le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt; reste, malgré la chaîne. La pomme se cale, le seau rentre, léger. Le sac pèse, grain près de la croûte. Le grain a parlé, très bas. Le goûter a un seau, sans chaîne ! La chaîne a failli tout garder. Une croûte garde l'ombre de la chaîne, près du grain. Le grain est là, tu le sens ? Oui, c'est celui de la buée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>La pomme dans le seau, quand la sangle est libre ! Nina attend que la chaîne se taise. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. La pomme se cale, le seau rentre, léger. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. Le goûter a un seau, sans chaîne ! La chaîne a failli tout garder. Une croûte garde l'ombre de la chaîne, près du grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>La pomme dans le seau, quand la sangle est libre ! Nina attend que la chaîne se taise. Le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt; reste, malgré la chaîne. La pomme se cale, le seau rentre, léger. Le sac pèse, grain près de la croûte. Le grain a parlé, très bas. Le goûter a un seau, sans chaîne ! La chaîne a failli tout garder. Une croûte garde l'ombre de la chaîne, près du grain. Le grain est là, tu le sens ? Oui, c'est celui de la buée. [pause]</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -15307,15 +15307,15 @@
         <is>
           <t>enfant-f|La pomme dans le seau, quand la sangle est libre !
 narrateur|Nina attend que la chaîne se taise.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Le grain de sel reste, malgré la chaîne.
 narrateur|La pomme se cale, le seau rentre, léger.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le sac pèse, grain près de la croûte.
 papa|Le grain a parlé, très bas.
 enfant-f|Le goûter a un seau, sans chaîne !
 maman|La chaîne a failli tout garder.
 narrateur|Une croûte garde l'ombre de la chaîne, près du grain.
-papa|Tu as vu le grain, sur le bouton ?
-enfant-f|Il était sur la vitre, à la cuisine.</t>
+papa|Le grain est là, tu le sens ?
+enfant-f|Oui, c'est celui de la buée.</t>
         </is>
       </c>
       <c r="AX76" t="inlineStr">
@@ -15530,17 +15530,17 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>La casquette pour ombrer le seau, dans le sac ! Nina décroche, puis pose la visière. Elle suit le grain de sel, jusqu'au bouton de bois. Le seau rentre, casquette dessus, léger. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. La visière a ombré, sans tirer ! La chaîne a failli tout garder. La visière ombre le seau, grain de sel au milieu. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>La casquette pour ombrer le seau, dans le sac ! Nina décroche, puis pose la visière. Elle suit le grain, de l'herbe au bois. Le seau rentre, casquette dessus, léger. Le bouton rentre, visière au milieu. Le grain a parlé, comme une lanterne. La visière a ombré, sans tirer ! La chaîne a failli tout garder. La visière ombre le seau, grain de sel au milieu. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La casquette pour ombrer le seau, dans le sac ! Nina décroche, puis pose la visière. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le seau rentre, casquette dessus, léger. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. La visière a ombré, sans tirer ! La chaîne a failli tout garder. La visière ombre le seau, grain de sel au milieu. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La casquette pour ombrer le seau, dans le sac ! Nina décroche, puis pose la visière. Elle suit le grain, de l'herbe au bois. Le seau rentre, casquette dessus, léger. Le bouton rentre, visière au milieu. Le grain a parlé, comme une lanterne. La visière a ombré, sans tirer ! La chaîne a failli tout garder. La visière ombre le seau, &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt; au milieu. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>La casquette pour ombrer le seau, dans le sac ! Nina décroche, puis pose la visière. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le seau rentre, casquette dessus, léger. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. La visière a ombré, sans tirer ! La chaîne a failli tout garder. La visière ombre le seau, grain de sel au milieu. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>La casquette pour ombrer le seau, dans le sac ! Nina décroche, puis pose la visière. Elle suit le grain, de l'herbe au bois. Le seau rentre, casquette dessus, léger. Le bouton rentre, visière au milieu. Le grain a parlé, comme une lanterne. La visière a ombré, sans tirer ! La chaîne a failli tout garder. La visière ombre le seau, &lt;emphasis&gt;grain de sel&lt;/emphasis&gt; au milieu. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit. [pause]</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -15676,15 +15676,15 @@
         <is>
           <t>enfant-f|La casquette pour ombrer le seau, dans le sac !
 narrateur|Nina décroche, puis pose la visière.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Elle suit le grain, de l'herbe au bois.
 narrateur|Le seau rentre, casquette dessus, léger.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le bouton rentre, visière au milieu.
 papa|Le grain a parlé, comme une lanterne.
 enfant-f|La visière a ombré, sans tirer !
 maman|La chaîne a failli tout garder.
 narrateur|La visière ombre le seau, grain de sel au milieu.
-papa|Tu as vu le grain, sur le bouton ?
-enfant-f|Il était sur la vitre, à la cuisine.</t>
+papa|Tu reconnais le grain, du verre ?
+enfant-f|Il a glissé du verre, tout petit.</t>
         </is>
       </c>
       <c r="AX78" t="inlineStr">
@@ -16293,17 +16293,17 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Je libère l'oreille, puis la gourde dans le sac ! Nina ouvre la chaîne, sans arracher. Elle suit le grain de sel, jusqu'au bouton de bois. Le doudou rentre, la gourde contre l'oreille. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. L'oreille est libre, et au nid ! La chaîne a failli tout garder. L'oreille du doudou sent l'herbe, sous le grain de sel. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>Je libère l'oreille, puis la gourde dans le sac ! Nina ouvre la chaîne, sans arracher. Nina libère l'oreille, puis voit le grain. Le doudou rentre, la gourde contre l'oreille. Le bois ferme, grain contre l'oreille. Le grain a parlé, sur le bois. L'oreille est libre, et au nid ! La chaîne a failli tout garder. L'oreille du doudou sent l'herbe, sous le grain de sel. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Je libère l'oreille, puis la gourde dans le sac ! Nina ouvre la chaîne, sans arracher. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le doudou rentre, la gourde contre l'oreille. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. L'oreille est libre, et au nid ! La chaîne a failli tout garder. L'oreille du doudou sent l'herbe, sous le grain de sel. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Je libère l'oreille, puis la gourde dans le sac ! Nina ouvre la chaîne, sans arracher. Nina libère l'oreille, puis voit le grain. Le doudou rentre, la gourde contre l'oreille. Le bois ferme, grain contre l'oreille. Le grain a parlé, sur le bois. L'oreille est libre, et au nid ! La chaîne a failli tout garder. L'oreille du doudou sent l'herbe, sous le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Je libère l'oreille, puis la gourde dans le sac ! Nina ouvre la chaîne, sans arracher. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le doudou rentre, la gourde contre l'oreille. Le bouton ferme, net, sur le grain. Le grain a parlé, sur le bois. L'oreille est libre, et au nid ! La chaîne a failli tout garder. L'oreille du doudou sent l'herbe, sous le grain de sel. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>Je libère l'oreille, puis la gourde dans le sac ! Nina ouvre la chaîne, sans arracher. Nina libère l'oreille, puis voit le grain. Le doudou rentre, la gourde contre l'oreille. Le bois ferme, grain contre l'oreille. Le grain a parlé, sur le bois. L'oreille est libre, et au nid ! La chaîne a failli tout garder. L'oreille du doudou sent l'herbe, sous le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
@@ -16439,9 +16439,9 @@
         <is>
           <t>enfant-f|Je libère l'oreille, puis la gourde dans le sac !
 narrateur|Nina ouvre la chaîne, sans arracher.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Nina libère l'oreille, puis voit le grain.
 narrateur|Le doudou rentre, la gourde contre l'oreille.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le bois ferme, grain contre l'oreille.
 papa|Le grain a parlé, sur le bois.
 enfant-f|L'oreille est libre, et au nid !
 maman|La chaîne a failli tout garder.
@@ -16666,17 +16666,17 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>La pomme pour réchauffer l'oreille, dans le sac ! Nina ouvre la chaîne, un maillon après l'autre. Elle suit le grain de sel, jusqu'au bouton de bois. Le doudou rentre, la pomme contre l'oreille. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. L'oreille a un goûter, maintenant ! La chaîne a failli tout garder. La pomme a réchauffé l'oreille, près du grain de sel. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>La pomme pour réchauffer l'oreille, dans le sac ! Nina ouvre la chaîne, un maillon après l'autre. Le grain de sel chauffe, sous son doigt. Le doudou rentre, la pomme contre l'oreille. Le bouton tient, grain près de la pomme. Le grain a parlé, très bas. L'oreille a un goûter, maintenant ! La chaîne a failli tout garder. La pomme a réchauffé l'oreille, près du grain de sel. Le grain est là, tu le sens ? Oui, c'est celui de la buée.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La pomme pour réchauffer l'oreille, dans le sac ! Nina ouvre la chaîne, un maillon après l'autre. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le doudou rentre, la pomme contre l'oreille. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. L'oreille a un goûter, maintenant ! La chaîne a failli tout garder. La pomme a réchauffé l'oreille, près du grain de sel. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La pomme pour réchauffer l'oreille, dans le sac ! Nina ouvre la chaîne, un maillon après l'autre. Le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt; chauffe, sous son doigt. Le doudou rentre, la pomme contre l'oreille. Le bouton tient, grain près de la pomme. Le grain a parlé, très bas. L'oreille a un goûter, maintenant ! La chaîne a failli tout garder. La pomme a réchauffé l'oreille, près du grain de sel. Le grain est là, tu le sens ? Oui, c'est celui de la buée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>La pomme pour réchauffer l'oreille, dans le sac ! Nina ouvre la chaîne, un maillon après l'autre. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le doudou rentre, la pomme contre l'oreille. Le bouton ferme, net, sur le grain. Le grain a parlé, très bas. L'oreille a un goûter, maintenant ! La chaîne a failli tout garder. La pomme a réchauffé l'oreille, près du grain de sel. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>La pomme pour réchauffer l'oreille, dans le sac ! Nina ouvre la chaîne, un maillon après l'autre. Le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt; chauffe, sous son doigt. Le doudou rentre, la pomme contre l'oreille. Le bouton tient, grain près de la pomme. Le grain a parlé, très bas. L'oreille a un goûter, maintenant ! La chaîne a failli tout garder. La pomme a réchauffé l'oreille, près du grain de sel. Le grain est là, tu le sens ? Oui, c'est celui de la buée. [pause]</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -16812,15 +16812,15 @@
         <is>
           <t>enfant-f|La pomme pour réchauffer l'oreille, dans le sac !
 narrateur|Nina ouvre la chaîne, un maillon après l'autre.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Le grain de sel chauffe, sous son doigt.
 narrateur|Le doudou rentre, la pomme contre l'oreille.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le bouton tient, grain près de la pomme.
 papa|Le grain a parlé, très bas.
 enfant-f|L'oreille a un goûter, maintenant !
 maman|La chaîne a failli tout garder.
 narrateur|La pomme a réchauffé l'oreille, près du grain de sel.
-papa|Tu as vu le grain, sur le bouton ?
-enfant-f|Il était sur la vitre, à la cuisine.</t>
+papa|Le grain est là, tu le sens ?
+enfant-f|Oui, c'est celui de la buée.</t>
         </is>
       </c>
       <c r="AX84" t="inlineStr">
@@ -17039,17 +17039,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>La casquette sur l'oreille, puis dans le sac ! Nina ouvre la chaîne, sans tirer le tissu. Elle suit le grain de sel, jusqu'au bouton de bois. Le doudou rentre, casquette sur l'oreille libre. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. Il a un chapeau, et un nid ! La chaîne a failli tout garder. Un dessin de chaîne reste sur la visière, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.</t>
+          <t>La casquette sur l'oreille, puis dans le sac ! Nina ouvre la chaîne, sans tirer le tissu. Elle pose le doigt au centre du bouton, sur le grain. Le doudou rentre, casquette sur l'oreille libre. Le sac se cale, grain sous le dessin. Le grain a parlé, comme une lanterne. Il a un chapeau, et un nid ! La chaîne a failli tout garder. Un dessin de chaîne reste sur la visière, sous le grain. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La casquette sur l'oreille, puis dans le sac ! Nina ouvre la chaîne, sans tirer le tissu. Elle suit le &lt;emphasis level="moderate"&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le doudou rentre, casquette sur l'oreille libre. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. Il a un chapeau, et un nid ! La chaîne a failli tout garder. Un dessin de chaîne reste sur la visière, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La casquette sur l'oreille, puis dans le sac ! Nina ouvre la chaîne, sans tirer le tissu. Elle pose le doigt au centre du bouton, sur le grain. Le doudou rentre, casquette sur l'oreille libre. Le sac se cale, grain sous le dessin. Le grain a parlé, comme une lanterne. Il a un chapeau, et un nid ! La chaîne a failli tout garder. Un dessin de chaîne reste sur la visière, sous le grain. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>La casquette sur l'oreille, puis dans le sac ! Nina ouvre la chaîne, sans tirer le tissu. Elle suit le &lt;emphasis&gt;grain de sel&lt;/emphasis&gt;, jusqu'au bouton de bois. Le doudou rentre, casquette sur l'oreille libre. Le bouton ferme, net, sur le grain. Le grain a parlé, comme une lanterne. Il a un chapeau, et un nid ! La chaîne a failli tout garder. Un dessin de chaîne reste sur la visière, sous le grain. Tu as vu le grain, sur le bouton ? Il était sur la vitre, à la cuisine. [pause]</t>
+          <t>La casquette sur l'oreille, puis dans le sac ! Nina ouvre la chaîne, sans tirer le tissu. Elle pose le doigt au centre du bouton, sur le grain. Le doudou rentre, casquette sur l'oreille libre. Le sac se cale, grain sous le dessin. Le grain a parlé, comme une lanterne. Il a un chapeau, et un nid ! La chaîne a failli tout garder. Un dessin de chaîne reste sur la visière, sous le grain. Tu reconnais le grain, du verre ? Il a glissé du verre, tout petit. [pause]</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -17185,15 +17185,15 @@
         <is>
           <t>enfant-f|La casquette sur l'oreille, puis dans le sac !
 narrateur|Nina ouvre la chaîne, sans tirer le tissu.
-narrateur|Elle suit le grain de sel, jusqu'au bouton de bois.
+narrateur|Elle pose le doigt au centre du bouton, sur le grain.
 narrateur|Le doudou rentre, casquette sur l'oreille libre.
-narrateur|Le bouton ferme, net, sur le grain.
+narrateur|Le sac se cale, grain sous le dessin.
 papa|Le grain a parlé, comme une lanterne.
 enfant-f|Il a un chapeau, et un nid !
 maman|La chaîne a failli tout garder.
 narrateur|Un dessin de chaîne reste sur la visière, sous le grain.
-papa|Tu as vu le grain, sur le bouton ?
-enfant-f|Il était sur la vitre, à la cuisine.</t>
+papa|Tu reconnais le grain, du verre ?
+enfant-f|Il a glissé du verre, tout petit.</t>
         </is>
       </c>
       <c r="AX86" t="inlineStr">
@@ -17406,7 +17406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17540,6 +17540,13 @@
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>